<commit_message>
Actualización de archivos JSON y scripts 05 de marzo 2026
</commit_message>
<xml_diff>
--- a/Alfa.xlsx
+++ b/Alfa.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="506">
   <si>
     <t>Asignado a</t>
   </si>
@@ -1684,10 +1684,12 @@
     <t>Cargue de archivos</t>
   </si>
   <si>
-    <t>09/02/2026 al 11/02/2026: Se está trabajando en el cargue de las diversas fuentes requeridas para la gestión de procesos jurídicos:
+    <t xml:space="preserve">09/02/2026 al 11/02/2026: Se está trabajando en el cargue de las diversas fuentes requeridas para la gestión de procesos jurídicos:
         Base siniestro y Bodega de datos.
         Cálculos y Consecutivos de Juntas.
-        Resumen de Pago de Siniestros.</t>
+        Resumen de Pago de Siniestros.
+25/02/2026: Refacción de Archivos y Formatos. Adaptación de archivos de acuerdo a los procesos de la unidad. Se enfrentaron retos técnicos por carga de archivos de alta capacidad (más de 40 GB).
+</t>
   </si>
   <si>
     <t>Img_2025_033</t>
@@ -1763,7 +1765,8 @@
     <t>Se requiere reestructurar la forma como se crea el cronograma actualmente</t>
   </si>
   <si>
-    <t>11/02/2026 - 17/02/2026 - 19/02/2026 - 20/02/2026: Cronograma: Este componente tiene uno de los impactos funcionales más altos. Se requiere reestructurar el planificador incorporando temáticas, permitiendo calendarios más flexibles y habilitando la generación masiva de órdenes de servicio a futuro, lo que cambia por completo la forma en que opera la planificación anual del área.</t>
+    <t>11/02/2026 - 17/02/2026 - 19/02/2026 - 20/02/2026: Cronograma: Este componente tiene uno de los impactos funcionales más altos. Se requiere reestructurar el planificador incorporando temáticas, permitiendo calendarios más flexibles y habilitando la generación masiva de órdenes de servicio a futuro, lo que cambia por completo la forma en que opera la planificación anual del área.
+23/02/2026: Rediseño integral del flujo para la creación de planes de trabajo, optimizando la entrada de datos.</t>
   </si>
   <si>
     <t>SST_2025_026</t>
@@ -1775,9 +1778,9 @@
     <t>Modificación en la creación y generación de ordenes de servicio</t>
   </si>
   <si>
-    <t xml:space="preserve">11/02/2026 - 17/02/2026 - 19/02/2026 - 20/02/2026: Pre-Orden de Servicio: Se ajusta la lógica de acuerdo con el nuevo flujo basado en temáticas y su integración con el cronograma y la acreditación de profesionales, afectando reglas, validaciones y la estructura de la pre-orden como tal. 
+    <t>11/02/2026 - 17/02/2026 - 19/02/2026 - 20/02/2026: Pre-Orden de Servicio: Se ajusta la lógica de acuerdo con el nuevo flujo basado en temáticas y su integración con el cronograma y la acreditación de profesionales, afectando reglas, validaciones y la estructura de la pre-orden como tal. 
         Notas Adicionales: Queda pendiente el impacto en informes y nuevos datos estadísticos requeridos por el cliente. Se terminó la creación y modificación de las agendas; queda pendiente la modificación de las agendas por actividad.
-</t>
+25/02/2026: Integración de la nueva funcionalidad para agendar órdenes de servicio (OS) directamente desde el plan de trabajo.</t>
   </si>
   <si>
     <t>Img_2025_034</t>
@@ -1824,6 +1827,66 @@
   </si>
   <si>
     <t>20/02/2026:         A las 22:00 horas, se procedió con la detención programada de los servicios Apache y PostgreSQL. Esta interrupción se realizó con el fin de facilitar las actividades de gestión de acceso privilegiado (PAM) ejecutadas por el equipo Alfa.</t>
+  </si>
+  <si>
+    <t>SST_2025_027</t>
+  </si>
+  <si>
+    <t>Plan de Trabajo ALFASST - Modulo de Edición</t>
+  </si>
+  <si>
+    <t>Se requiere que los datos registrados en las OS puedan ser editados</t>
+  </si>
+  <si>
+    <t>24/02/2026: Ajuste y optimización de la funcionalidad para modificar registros existentes de forma fluida.</t>
+  </si>
+  <si>
+    <t>SST_2025_028</t>
+  </si>
+  <si>
+    <t>Plan de Trabajo ALFASST - Logica de Validaciones</t>
+  </si>
+  <si>
+    <t>Se requiere que las OS sean agendadas correctamente</t>
+  </si>
+  <si>
+    <t>26/02/2026: Implementación de reglas técnicas y de negocio para asegurar que las agendas se generen sin errores ni traslapes.</t>
+  </si>
+  <si>
+    <t>PRV_2025_045</t>
+  </si>
+  <si>
+    <t>Configuración de Servidor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajustes de infraestructura en el servidor para cargar archivos </t>
+  </si>
+  <si>
+    <t>26/02/2026: Ajustes en la infraestructura para evitar caídas y detenciones del sistema causadas por el volumen excesivo de los archivos cargados.</t>
+  </si>
+  <si>
+    <t>PRV_2025_046</t>
+  </si>
+  <si>
+    <t>Acompañamiento en sesiòn de unidad</t>
+  </si>
+  <si>
+    <t>Sesión de validaciones</t>
+  </si>
+  <si>
+    <t>27/02/2026: Sesión de validación sobre la carga de archivos. Se planteó nuevamente la necesidad técnica de integrar la base de datos para optimizar los procesos.</t>
+  </si>
+  <si>
+    <t>PRV_2025_047</t>
+  </si>
+  <si>
+    <t>Tablero de Control - Control de cambios</t>
+  </si>
+  <si>
+    <t>Ajuste de visualizaciòn de datos</t>
+  </si>
+  <si>
+    <t>27/02/2026: Corrección del error en el tablero de control que impedía la generación del año en vigencia, normalizando los reportes actuales.</t>
   </si>
 </sst>
 </file>
@@ -2770,7 +2833,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla" displayName="Tabla" ref="A1:S136">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla" displayName="Tabla" ref="A1:S141">
   <tableColumns count="19">
     <tableColumn id="1" name="Asignado a"/>
     <tableColumn id="2" name="# REQ"/>
@@ -3062,7 +3125,7 @@
   <sheetPr>
     <tabColor rgb="FFCC0000"/>
   </sheetPr>
-  <dimension ref="A1:S1054"/>
+  <dimension ref="A1:S1060"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.125" style="14" customWidth="1"/>
@@ -9067,7 +9130,7 @@
       NETWORKDAYS(J105,L105,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="N105" s="84"/>
       <c r="O105" s="84"/>
@@ -10047,7 +10110,7 @@
       NETWORKDAYS(J122,L122,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="N122" s="68"/>
       <c r="O122" s="68"/>
@@ -10196,7 +10259,7 @@
         <v>369</v>
       </c>
       <c r="G125" s="78">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="H125" s="21">
         <f>IF(OR(J125="",K125="",K125&lt;J125),0,NETWORKDAYS(J125,K125,[1]fESTIVOS!$A$2:$A$53))</f>
@@ -10217,7 +10280,7 @@
       NETWORKDAYS(J125,L125,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="N125" s="68"/>
       <c r="O125" s="68"/>
@@ -10387,7 +10450,7 @@
       NETWORKDAYS(J128,L128,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="N128" s="84"/>
       <c r="O128" s="84"/>
@@ -10441,7 +10504,7 @@
       NETWORKDAYS(J129,L129,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="N129" s="84"/>
       <c r="O129" s="84"/>
@@ -10495,7 +10558,7 @@
       NETWORKDAYS(J130,L130,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="N130" s="84"/>
       <c r="O130" s="84"/>
@@ -10549,7 +10612,7 @@
       NETWORKDAYS(J131,L131,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="N131" s="84"/>
       <c r="O131" s="84"/>
@@ -10579,14 +10642,14 @@
         <v>105</v>
       </c>
       <c r="F132" s="91" t="s">
-        <v>369</v>
+        <v>23</v>
       </c>
       <c r="G132" s="83">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="H132" s="21">
         <f>IF(OR(J133="",K132="",K132&lt;J133),0,NETWORKDAYS(J133,K132,[1]fESTIVOS!$A$2:$A$53))</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I132" s="87">
         <v>46064</v>
@@ -10594,13 +10657,17 @@
       <c r="J132" s="73">
         <v>46064</v>
       </c>
-      <c r="K132" s="73"/>
-      <c r="L132" s="73"/>
+      <c r="K132" s="73">
+        <v>46076</v>
+      </c>
+      <c r="L132" s="73">
+        <v>46076</v>
+      </c>
       <c r="M132" s="25">
-        <f ca="1">IF(OR(J133="",AND(L132="",TODAY()&lt;J133),AND(L132&lt;&gt;"",L132&lt;J133)),0,
+        <f ca="1">IF(OR(J132="",AND(L132="",TODAY()&lt;J132),AND(L132&lt;&gt;"",L132&lt;J132)),0,
    IF(L132="",
-      NETWORKDAYS(J133,TODAY(),[1]fESTIVOS!$A$2:$A$53),
-      NETWORKDAYS(J133,L132,[1]fESTIVOS!$A$2:$A$53)
+      NETWORKDAYS(J132,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J132,L132,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
         <v>9</v>
@@ -10633,14 +10700,14 @@
         <v>105</v>
       </c>
       <c r="F133" s="91" t="s">
-        <v>369</v>
+        <v>23</v>
       </c>
       <c r="G133" s="83">
-        <v>50</v>
-      </c>
-      <c r="H133" s="21" t="e">
-        <f>IF(OR(#REF!="",K133="",K133&lt;#REF!),0,NETWORKDAYS(#REF!,K133,[1]fESTIVOS!$A$2:$A$53))</f>
-        <v>#REF!</v>
+        <v>100</v>
+      </c>
+      <c r="H133" s="21">
+        <f>IF(OR(J134="",K133="",K133&lt;J134),0,NETWORKDAYS(J134,K133,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>6</v>
       </c>
       <c r="I133" s="87">
         <v>46064</v>
@@ -10648,16 +10715,20 @@
       <c r="J133" s="73">
         <v>46064</v>
       </c>
-      <c r="K133" s="73"/>
-      <c r="L133" s="73"/>
-      <c r="M133" s="25" t="e">
-        <f ca="1">IF(OR(#REF!="",AND(L133="",TODAY()&lt;#REF!),AND(L133&lt;&gt;"",L133&lt;#REF!)),0,
+      <c r="K133" s="73">
+        <v>46078</v>
+      </c>
+      <c r="L133" s="73">
+        <v>46078</v>
+      </c>
+      <c r="M133" s="25">
+        <f ca="1">IF(OR(J133="",AND(L133="",TODAY()&lt;J133),AND(L133&lt;&gt;"",L133&lt;J133)),0,
    IF(L133="",
-      NETWORKDAYS(#REF!,TODAY(),[1]fESTIVOS!$A$2:$A$53),
-      NETWORKDAYS(#REF!,L133,[1]fESTIVOS!$A$2:$A$53)
-   )
-)</f>
-        <v>#REF!</v>
+      NETWORKDAYS(J133,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J133,L133,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>11</v>
       </c>
       <c r="N133" s="84"/>
       <c r="O133" s="84"/>
@@ -10844,11 +10915,296 @@
       </c>
       <c r="S136" s="76"/>
     </row>
-    <row r="137" spans="1:19" ht="29.25" customHeight="1"/>
-    <row r="138" spans="1:19" ht="29.25" customHeight="1"/>
-    <row r="139" spans="1:19" ht="29.25" customHeight="1"/>
-    <row r="140" spans="1:19" ht="29.25" customHeight="1"/>
-    <row r="141" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="137" spans="1:19" ht="29.25" customHeight="1">
+      <c r="A137" s="80" t="s">
+        <v>19</v>
+      </c>
+      <c r="B137" s="63" t="s">
+        <v>486</v>
+      </c>
+      <c r="C137" s="81" t="s">
+        <v>487</v>
+      </c>
+      <c r="D137" s="92" t="s">
+        <v>488</v>
+      </c>
+      <c r="E137" s="63" t="s">
+        <v>105</v>
+      </c>
+      <c r="F137" s="91" t="s">
+        <v>23</v>
+      </c>
+      <c r="G137" s="83">
+        <v>100</v>
+      </c>
+      <c r="H137" s="21">
+        <f>IF(OR(J137="",K137="",K137&lt;J137),0,NETWORKDAYS(J137,K137,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I137" s="87">
+        <v>46077</v>
+      </c>
+      <c r="J137" s="73">
+        <v>46077</v>
+      </c>
+      <c r="K137" s="73">
+        <v>46077</v>
+      </c>
+      <c r="L137" s="73">
+        <v>46077</v>
+      </c>
+      <c r="M137" s="25">
+        <f ca="1">IF(OR(J137="",AND(L137="",TODAY()&lt;J137),AND(L137&lt;&gt;"",L137&lt;J137)),0,
+   IF(L137="",
+      NETWORKDAYS(J137,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J137,L137,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N137" s="84"/>
+      <c r="O137" s="84"/>
+      <c r="P137" s="85"/>
+      <c r="Q137" s="97" t="s">
+        <v>489</v>
+      </c>
+      <c r="R137" s="71" t="s">
+        <v>25</v>
+      </c>
+      <c r="S137" s="70"/>
+    </row>
+    <row r="138" spans="1:19" ht="29.25" customHeight="1">
+      <c r="A138" s="80" t="s">
+        <v>19</v>
+      </c>
+      <c r="B138" s="63" t="s">
+        <v>490</v>
+      </c>
+      <c r="C138" s="81" t="s">
+        <v>491</v>
+      </c>
+      <c r="D138" s="92" t="s">
+        <v>492</v>
+      </c>
+      <c r="E138" s="63" t="s">
+        <v>105</v>
+      </c>
+      <c r="F138" s="91" t="s">
+        <v>23</v>
+      </c>
+      <c r="G138" s="83">
+        <v>100</v>
+      </c>
+      <c r="H138" s="21">
+        <f>IF(OR(J138="",K138="",K138&lt;J138),0,NETWORKDAYS(J138,K138,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I138" s="87">
+        <v>46079</v>
+      </c>
+      <c r="J138" s="73">
+        <v>46079</v>
+      </c>
+      <c r="K138" s="73">
+        <v>46079</v>
+      </c>
+      <c r="L138" s="73">
+        <v>46079</v>
+      </c>
+      <c r="M138" s="25">
+        <f ca="1">IF(OR(J138="",AND(L138="",TODAY()&lt;J138),AND(L138&lt;&gt;"",L138&lt;J138)),0,
+   IF(L138="",
+      NETWORKDAYS(J138,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J138,L138,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N138" s="84"/>
+      <c r="O138" s="84"/>
+      <c r="P138" s="85"/>
+      <c r="Q138" s="97" t="s">
+        <v>493</v>
+      </c>
+      <c r="R138" s="71" t="s">
+        <v>25</v>
+      </c>
+      <c r="S138" s="70"/>
+    </row>
+    <row r="139" spans="1:19" ht="29.25" customHeight="1">
+      <c r="A139" s="88" t="s">
+        <v>19</v>
+      </c>
+      <c r="B139" s="63" t="s">
+        <v>494</v>
+      </c>
+      <c r="C139" s="89" t="s">
+        <v>495</v>
+      </c>
+      <c r="D139" s="93" t="s">
+        <v>496</v>
+      </c>
+      <c r="E139" s="77" t="s">
+        <v>22</v>
+      </c>
+      <c r="F139" s="90" t="s">
+        <v>23</v>
+      </c>
+      <c r="G139" s="78">
+        <v>100</v>
+      </c>
+      <c r="H139" s="21">
+        <f>IF(OR(J139="",K139="",K139&lt;J139),0,NETWORKDAYS(J139,K139,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I139" s="87">
+        <v>46079</v>
+      </c>
+      <c r="J139" s="73">
+        <v>46079</v>
+      </c>
+      <c r="K139" s="73">
+        <v>46079</v>
+      </c>
+      <c r="L139" s="73">
+        <v>46079</v>
+      </c>
+      <c r="M139" s="25">
+        <f ca="1">IF(OR(J139="",AND(L139="",TODAY()&lt;J139),AND(L139&lt;&gt;"",L139&lt;J139)),0,
+   IF(L139="",
+      NETWORKDAYS(J139,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J139,L139,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N139" s="68"/>
+      <c r="O139" s="68"/>
+      <c r="P139" s="69"/>
+      <c r="Q139" s="96" t="s">
+        <v>497</v>
+      </c>
+      <c r="R139" s="79" t="s">
+        <v>25</v>
+      </c>
+      <c r="S139" s="76"/>
+    </row>
+    <row r="140" spans="1:19" ht="29.25" customHeight="1">
+      <c r="A140" s="88" t="s">
+        <v>19</v>
+      </c>
+      <c r="B140" s="63" t="s">
+        <v>498</v>
+      </c>
+      <c r="C140" s="89" t="s">
+        <v>499</v>
+      </c>
+      <c r="D140" s="93" t="s">
+        <v>500</v>
+      </c>
+      <c r="E140" s="77" t="s">
+        <v>22</v>
+      </c>
+      <c r="F140" s="90" t="s">
+        <v>23</v>
+      </c>
+      <c r="G140" s="78">
+        <v>100</v>
+      </c>
+      <c r="H140" s="21">
+        <f>IF(OR(J140="",K140="",K140&lt;J140),0,NETWORKDAYS(J140,K140,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I140" s="87">
+        <v>46080</v>
+      </c>
+      <c r="J140" s="73">
+        <v>46080</v>
+      </c>
+      <c r="K140" s="73">
+        <v>46080</v>
+      </c>
+      <c r="L140" s="73">
+        <v>46080</v>
+      </c>
+      <c r="M140" s="25">
+        <f ca="1">IF(OR(J140="",AND(L140="",TODAY()&lt;J140),AND(L140&lt;&gt;"",L140&lt;J140)),0,
+   IF(L140="",
+      NETWORKDAYS(J140,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J140,L140,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N140" s="68"/>
+      <c r="O140" s="68"/>
+      <c r="P140" s="69"/>
+      <c r="Q140" s="96" t="s">
+        <v>501</v>
+      </c>
+      <c r="R140" s="79" t="s">
+        <v>25</v>
+      </c>
+      <c r="S140" s="76"/>
+    </row>
+    <row r="141" spans="1:19" ht="29.25" customHeight="1">
+      <c r="A141" s="88" t="s">
+        <v>19</v>
+      </c>
+      <c r="B141" s="63" t="s">
+        <v>502</v>
+      </c>
+      <c r="C141" s="89" t="s">
+        <v>503</v>
+      </c>
+      <c r="D141" s="93" t="s">
+        <v>504</v>
+      </c>
+      <c r="E141" s="77" t="s">
+        <v>22</v>
+      </c>
+      <c r="F141" s="90" t="s">
+        <v>23</v>
+      </c>
+      <c r="G141" s="78">
+        <v>100</v>
+      </c>
+      <c r="H141" s="21">
+        <f>IF(OR(J141="",K141="",K141&lt;J141),0,NETWORKDAYS(J141,K141,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I141" s="87">
+        <v>46080</v>
+      </c>
+      <c r="J141" s="73">
+        <v>46080</v>
+      </c>
+      <c r="K141" s="73">
+        <v>46080</v>
+      </c>
+      <c r="L141" s="73">
+        <v>46080</v>
+      </c>
+      <c r="M141" s="25">
+        <f ca="1">IF(OR(J141="",AND(L141="",TODAY()&lt;J141),AND(L141&lt;&gt;"",L141&lt;J141)),0,
+   IF(L141="",
+      NETWORKDAYS(J141,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J141,L141,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N141" s="68"/>
+      <c r="O141" s="68"/>
+      <c r="P141" s="69"/>
+      <c r="Q141" s="96" t="s">
+        <v>505</v>
+      </c>
+      <c r="R141" s="79" t="s">
+        <v>25</v>
+      </c>
+      <c r="S141" s="76"/>
+    </row>
     <row r="142" spans="1:19" ht="29.25" customHeight="1"/>
     <row r="143" spans="1:19" ht="29.25" customHeight="1"/>
     <row r="144" spans="1:19" ht="29.25" customHeight="1"/>
@@ -11762,18 +12118,24 @@
     <row r="1052" ht="29.25" customHeight="1"/>
     <row r="1053" ht="29.25" customHeight="1"/>
     <row r="1054" ht="29.25" customHeight="1"/>
+    <row r="1055" ht="29.25" customHeight="1"/>
+    <row r="1056" ht="29.25" customHeight="1"/>
+    <row r="1057" ht="29.25" customHeight="1"/>
+    <row r="1058" ht="29.25" customHeight="1"/>
+    <row r="1059" ht="29.25" customHeight="1"/>
+    <row r="1060" ht="29.25" customHeight="1"/>
   </sheetData>
-  <conditionalFormatting sqref="B2:B137">
+  <conditionalFormatting sqref="B2:B142">
     <cfRule type="expression" dxfId="0" priority="2">
-      <formula>COUNTIF($B$2:$B$136,B2)&gt;1</formula>
+      <formula>COUNTIF($B$2:$B$141,B2)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="1" showDropDown="1" sqref="R2:R136"/>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:L136 O2:P136">
+    <dataValidation allowBlank="1" showDropDown="1" sqref="R2:R141"/>
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:L141 O2:P141">
       <formula1>OR(NOT(ISERROR(DATEVALUE(I2))), AND(ISNUMBER(I2), LEFT(CELL("format", I2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F136">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F141">
       <formula1>"FINALIZADO,EN PROCESO,PAUSADO,EN TEST,PENDIENTE,PRUEBAS CLIENTE,PENDIENTE CLIENTE,PRUEBAS IMAGINE,PASO A PRODUCCION"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Actualización de archivos JSON y scripts 06 de marzo 2026
</commit_message>
<xml_diff>
--- a/Alfa.xlsx
+++ b/Alfa.xlsx
@@ -17,6 +17,9 @@
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EN PROCESO (Alfa)'!$A$1:$S$147</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -27,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1143" uniqueCount="527">
   <si>
     <t>Asignado a</t>
   </si>
@@ -1717,7 +1720,8 @@
     <t>Modificación en el tarifario</t>
   </si>
   <si>
-    <t>11/02/2026 - 17/02/2026 - 19/02/2026 - 20/02/2026: Actividades (Temáticas): Se ejecuta un cambio estructural del modelo de tarifación, pasando del esquema tradicional basado en actividades individuales a un concepto de temáticas, las cuales agrupan programas y actividades asociadas a un costo determinado. Avance 90%. Queda pendiente realizar despliegue y pruebas en el ambiente de PT, para posterior desplegar al ambiente de QA y que el cliente realice las actividades.</t>
+    <t>11/02/2026 - 17/02/2026 - 19/02/2026 - 20/02/2026: Actividades (Temáticas): Se ejecuta un cambio estructural del modelo de tarifación, pasando del esquema tradicional basado en actividades individuales a un concepto de temáticas, las cuales agrupan programas y actividades asociadas a un costo determinado. Avance 90%. Queda pendiente realizar despliegue y pruebas en el ambiente de PT, para posterior desplegar al ambiente de QA y que el cliente realice las actividades.
+25/02/2026: Se finaliza desarrollo y despliegue en ambientes de pruebas y producciòn</t>
   </si>
   <si>
     <t>SST_2025_022</t>
@@ -1729,7 +1733,8 @@
     <t>Modificación en la asignación de productos y tarifas a los proveedores</t>
   </si>
   <si>
-    <t>11/02/2026 - 17/02/2026 - 19/02/2026 - 20/02/2026: Administrador – Proveedor: Se ajusta la forma en que se asignan los productos y tarifas a los proveedores, alineándola al nuevo esquema por temáticas, lo que modifica reglas anteriores y requiere reconfigurar relaciones internas del sistema. Avance 90%. Queda pendiente realizar despliegue y pruebas en el ambiente de PT, para posterior desplegar al ambiente de QA y que el cliente realice las actividades.</t>
+    <t>11/02/2026 - 17/02/2026 - 19/02/2026 - 20/02/2026: Administrador – Proveedor: Se ajusta la forma en que se asignan los productos y tarifas a los proveedores, alineándola al nuevo esquema por temáticas, lo que modifica reglas anteriores y requiere reconfigurar relaciones internas del sistema. Avance 90%. Queda pendiente realizar despliegue y pruebas en el ambiente de PT, para posterior desplegar al ambiente de QA y que el cliente realice las actividades.
+26/02/2026: Se finaliza desarrollo y despliegue en ambientes de pruebas y producciòn</t>
   </si>
   <si>
     <t>SST_2025_023</t>
@@ -1753,7 +1758,8 @@
     <t>Modificación en la selección de sedes y creación de campo ciudad</t>
   </si>
   <si>
-    <t>11/02/2026 - 17/02/2026 - 19/02/2026 - 20/02/2026: Sedes: Se ajustó para que solo se permita una sede principal; al momento de generar un cronograma de trabajo, solo se tendrá en cuenta la principal y las demás sedes se deshabilitarán del sistema actual. Posteriormente, en la programación de las órdenes, se agregó el campo "ciudad" para mejorar la trazabilidad, normalización de datos y capacidades de gestión. Avance 90%. Queda pendiente realizar despliegue y pruebas en el ambiente de PT, para posterior desplegar al ambiente de QA y que el cliente realice las actividades.</t>
+    <t>11/02/2026 - 17/02/2026 - 19/02/2026 - 20/02/2026: Sedes: Se ajustó para que solo se permita una sede principal; al momento de generar un cronograma de trabajo, solo se tendrá en cuenta la principal y las demás sedes se deshabilitarán del sistema actual. Posteriormente, en la programación de las órdenes, se agregó el campo "ciudad" para mejorar la trazabilidad, normalización de datos y capacidades de gestión. Avance 90%. Queda pendiente realizar despliegue y pruebas en el ambiente de PT, para posterior desplegar al ambiente de QA y que el cliente realice las actividades.
+27/02/2026: Se finaliza desarrollo y despliegue en ambientes de pruebas y producciòn</t>
   </si>
   <si>
     <t>SST_2025_025</t>
@@ -1887,6 +1893,69 @@
   </si>
   <si>
     <t>27/02/2026: Corrección del error en el tablero de control que impedía la generación del año en vigencia, normalizando los reportes actuales.</t>
+  </si>
+  <si>
+    <t>SST_2025_029</t>
+  </si>
+  <si>
+    <t>Plan de Trabajo ALFASST - Ordenes de Servicio</t>
+  </si>
+  <si>
+    <t>Tarea Programada de Agendamiento.</t>
+  </si>
+  <si>
+    <t>02/03/2026 - 03/03/2026: Desarrollo del proceso automático para la generación masiva de órdenes de servicio, sincronizada con la agenda programada.</t>
+  </si>
+  <si>
+    <t>SST_2025_030</t>
+  </si>
+  <si>
+    <t>Plan de Trabajo ALFASST - Optimización Integral (CRUD)</t>
+  </si>
+  <si>
+    <t>Creación, Edición, Modificación y Eliminación</t>
+  </si>
+  <si>
+    <t>04/03/2026: Fortalecimiento de procesos (Creación, Edición, Modificación y Eliminación). Ajuste de lógica para permitir la edición de planes cuando no existan agendas previas.</t>
+  </si>
+  <si>
+    <t>SST_2025_031</t>
+  </si>
+  <si>
+    <t>Plan de Trabajo ALFASST - Asignación actividades</t>
+  </si>
+  <si>
+    <t>Mejora Visual de Asignación.</t>
+  </si>
+  <si>
+    <t>04/03/2026: Optimización de la interfaz (UI) para la asignación de actividades, facilitando la gestión visual.</t>
+  </si>
+  <si>
+    <t>PRV_2025_048</t>
+  </si>
+  <si>
+    <t>Reservas</t>
+  </si>
+  <si>
+    <t>Nuevo Módulo de Carga (Reservas).</t>
+  </si>
+  <si>
+    <t>03/03/2026 al 05/03/2026: Creación del módulo para carga masiva de reservas con formatos específicos. Se implementó un reporte dinámico para exportar información por tipo de formato.</t>
+  </si>
+  <si>
+    <t>PRV_2025_049</t>
+  </si>
+  <si>
+    <t>Optimización de Importación Masiva.</t>
+  </si>
+  <si>
+    <t>05/03/2026: Se eliminó el conteo de registros en caliente al adjuntar archivos, logrando una carga mucho más rápida y eficiente.</t>
+  </si>
+  <si>
+    <t>PRV_2025_050</t>
+  </si>
+  <si>
+    <t>06/03/2026: Pruebas finales para validar las mejoras, asegurando que la calidad de la información cumpla con las necesidades operativas de la unidad.</t>
   </si>
 </sst>
 </file>
@@ -2833,7 +2902,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla" displayName="Tabla" ref="A1:S141">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla" displayName="Tabla" ref="A1:S147">
+  <autoFilter ref="A1:S147"/>
   <tableColumns count="19">
     <tableColumn id="1" name="Asignado a"/>
     <tableColumn id="2" name="# REQ"/>
@@ -3125,7 +3195,7 @@
   <sheetPr>
     <tabColor rgb="FFCC0000"/>
   </sheetPr>
-  <dimension ref="A1:S1060"/>
+  <dimension ref="A1:S1066"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.125" style="14" customWidth="1"/>
@@ -9130,7 +9200,7 @@
       NETWORKDAYS(J105,L105,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N105" s="84"/>
       <c r="O105" s="84"/>
@@ -10110,7 +10180,7 @@
       NETWORKDAYS(J122,L122,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="N122" s="68"/>
       <c r="O122" s="68"/>
@@ -10280,7 +10350,7 @@
       NETWORKDAYS(J125,L125,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="N125" s="68"/>
       <c r="O125" s="68"/>
@@ -10426,14 +10496,14 @@
         <v>105</v>
       </c>
       <c r="F128" s="91" t="s">
-        <v>369</v>
+        <v>23</v>
       </c>
       <c r="G128" s="83">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="H128" s="21">
         <f>IF(OR(J128="",K128="",K128&lt;J128),0,NETWORKDAYS(J128,K128,[1]fESTIVOS!$A$2:$A$53))</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I128" s="87">
         <v>46064</v>
@@ -10441,8 +10511,12 @@
       <c r="J128" s="73">
         <v>46064</v>
       </c>
-      <c r="K128" s="73"/>
-      <c r="L128" s="73"/>
+      <c r="K128" s="73">
+        <v>46078</v>
+      </c>
+      <c r="L128" s="73">
+        <v>46078</v>
+      </c>
       <c r="M128" s="25">
         <f ca="1">IF(OR(J128="",AND(L128="",TODAY()&lt;J128),AND(L128&lt;&gt;"",L128&lt;J128)),0,
    IF(L128="",
@@ -10450,7 +10524,7 @@
       NETWORKDAYS(J128,L128,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="N128" s="84"/>
       <c r="O128" s="84"/>
@@ -10480,14 +10554,14 @@
         <v>105</v>
       </c>
       <c r="F129" s="91" t="s">
-        <v>369</v>
+        <v>23</v>
       </c>
       <c r="G129" s="83">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="H129" s="21">
         <f>IF(OR(J129="",K129="",K129&lt;J129),0,NETWORKDAYS(J129,K129,[1]fESTIVOS!$A$2:$A$53))</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I129" s="87">
         <v>46064</v>
@@ -10495,8 +10569,12 @@
       <c r="J129" s="73">
         <v>46064</v>
       </c>
-      <c r="K129" s="73"/>
-      <c r="L129" s="73"/>
+      <c r="K129" s="73">
+        <v>46079</v>
+      </c>
+      <c r="L129" s="73">
+        <v>46079</v>
+      </c>
       <c r="M129" s="25">
         <f ca="1">IF(OR(J129="",AND(L129="",TODAY()&lt;J129),AND(L129&lt;&gt;"",L129&lt;J129)),0,
    IF(L129="",
@@ -10504,7 +10582,7 @@
       NETWORKDAYS(J129,L129,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="N129" s="84"/>
       <c r="O129" s="84"/>
@@ -10558,7 +10636,7 @@
       NETWORKDAYS(J130,L130,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="N130" s="84"/>
       <c r="O130" s="84"/>
@@ -10588,14 +10666,14 @@
         <v>105</v>
       </c>
       <c r="F131" s="91" t="s">
-        <v>369</v>
+        <v>23</v>
       </c>
       <c r="G131" s="83">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="H131" s="21">
         <f>IF(OR(J131="",K131="",K131&lt;J131),0,NETWORKDAYS(J131,K131,[1]fESTIVOS!$A$2:$A$53))</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I131" s="87">
         <v>46064</v>
@@ -10603,8 +10681,12 @@
       <c r="J131" s="73">
         <v>46064</v>
       </c>
-      <c r="K131" s="73"/>
-      <c r="L131" s="73"/>
+      <c r="K131" s="73">
+        <v>46080</v>
+      </c>
+      <c r="L131" s="73">
+        <v>46080</v>
+      </c>
       <c r="M131" s="25">
         <f ca="1">IF(OR(J131="",AND(L131="",TODAY()&lt;J131),AND(L131&lt;&gt;"",L131&lt;J131)),0,
    IF(L131="",
@@ -10612,7 +10694,7 @@
       NETWORKDAYS(J131,L131,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N131" s="84"/>
       <c r="O131" s="84"/>
@@ -10664,10 +10746,10 @@
         <v>46076</v>
       </c>
       <c r="M132" s="25">
-        <f ca="1">IF(OR(J132="",AND(L132="",TODAY()&lt;J132),AND(L132&lt;&gt;"",L132&lt;J132)),0,
+        <f ca="1">IF(OR(J133="",AND(L132="",TODAY()&lt;J133),AND(L132&lt;&gt;"",L132&lt;J133)),0,
    IF(L132="",
-      NETWORKDAYS(J132,TODAY(),[1]fESTIVOS!$A$2:$A$53),
-      NETWORKDAYS(J132,L132,[1]fESTIVOS!$A$2:$A$53)
+      NETWORKDAYS(J133,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J133,L132,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
         <v>9</v>
@@ -10722,13 +10804,13 @@
         <v>46078</v>
       </c>
       <c r="M133" s="25">
-        <f ca="1">IF(OR(J133="",AND(L133="",TODAY()&lt;J133),AND(L133&lt;&gt;"",L133&lt;J133)),0,
+        <f ca="1">IF(OR(J134="",AND(L133="",TODAY()&lt;J134),AND(L133&lt;&gt;"",L133&lt;J134)),0,
    IF(L133="",
-      NETWORKDAYS(J133,TODAY(),[1]fESTIVOS!$A$2:$A$53),
-      NETWORKDAYS(J133,L133,[1]fESTIVOS!$A$2:$A$53)
-   )
-)</f>
-        <v>11</v>
+      NETWORKDAYS(J134,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J134,L133,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>6</v>
       </c>
       <c r="N133" s="84"/>
       <c r="O133" s="84"/>
@@ -10764,8 +10846,8 @@
         <v>100</v>
       </c>
       <c r="H134" s="21">
-        <f>IF(OR(J134="",K134="",K134&lt;J134),0,NETWORKDAYS(J134,K134,[1]fESTIVOS!$A$2:$A$53))</f>
-        <v>1</v>
+        <f>IF(OR(J135="",K134="",K134&lt;J135),0,NETWORKDAYS(J135,K134,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>0</v>
       </c>
       <c r="I134" s="94">
         <v>46071</v>
@@ -10780,13 +10862,13 @@
         <v>46071</v>
       </c>
       <c r="M134" s="25">
-        <f ca="1">IF(OR(J134="",AND(L134="",TODAY()&lt;J134),AND(L134&lt;&gt;"",L134&lt;J134)),0,
+        <f ca="1">IF(OR(J135="",AND(L134="",TODAY()&lt;J135),AND(L134&lt;&gt;"",L134&lt;J135)),0,
    IF(L134="",
-      NETWORKDAYS(J134,TODAY(),[1]fESTIVOS!$A$2:$A$53),
-      NETWORKDAYS(J134,L134,[1]fESTIVOS!$A$2:$A$53)
-   )
-)</f>
-        <v>1</v>
+      NETWORKDAYS(J135,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J135,L134,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
       </c>
       <c r="N134" s="68"/>
       <c r="O134" s="68"/>
@@ -10822,7 +10904,7 @@
         <v>100</v>
       </c>
       <c r="H135" s="21">
-        <f>IF(OR(J135="",K135="",K135&lt;J135),0,NETWORKDAYS(J135,K135,[1]fESTIVOS!$A$2:$A$53))</f>
+        <f>IF(OR(J136="",K135="",K135&lt;J136),0,NETWORKDAYS(J136,K135,[1]fESTIVOS!$A$2:$A$53))</f>
         <v>1</v>
       </c>
       <c r="I135" s="94">
@@ -10838,10 +10920,10 @@
         <v>46073</v>
       </c>
       <c r="M135" s="25">
-        <f ca="1">IF(OR(J135="",AND(L135="",TODAY()&lt;J135),AND(L135&lt;&gt;"",L135&lt;J135)),0,
+        <f ca="1">IF(OR(J136="",AND(L135="",TODAY()&lt;J136),AND(L135&lt;&gt;"",L135&lt;J136)),0,
    IF(L135="",
-      NETWORKDAYS(J135,TODAY(),[1]fESTIVOS!$A$2:$A$53),
-      NETWORKDAYS(J135,L135,[1]fESTIVOS!$A$2:$A$53)
+      NETWORKDAYS(J136,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J136,L135,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
         <v>1</v>
@@ -10880,8 +10962,8 @@
         <v>100</v>
       </c>
       <c r="H136" s="21">
-        <f>IF(OR(J136="",K136="",K136&lt;J136),0,NETWORKDAYS(J136,K136,[1]fESTIVOS!$A$2:$A$53))</f>
-        <v>1</v>
+        <f>IF(OR(J137="",K136="",K136&lt;J137),0,NETWORKDAYS(J137,K136,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>0</v>
       </c>
       <c r="I136" s="94">
         <v>46073</v>
@@ -10896,13 +10978,13 @@
         <v>46073</v>
       </c>
       <c r="M136" s="25">
-        <f ca="1">IF(OR(J136="",AND(L136="",TODAY()&lt;J136),AND(L136&lt;&gt;"",L136&lt;J136)),0,
+        <f ca="1">IF(OR(J137="",AND(L136="",TODAY()&lt;J137),AND(L136&lt;&gt;"",L136&lt;J137)),0,
    IF(L136="",
-      NETWORKDAYS(J136,TODAY(),[1]fESTIVOS!$A$2:$A$53),
-      NETWORKDAYS(J136,L136,[1]fESTIVOS!$A$2:$A$53)
-   )
-)</f>
-        <v>1</v>
+      NETWORKDAYS(J137,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J137,L136,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
       </c>
       <c r="N136" s="68"/>
       <c r="O136" s="68"/>
@@ -10938,8 +11020,8 @@
         <v>100</v>
       </c>
       <c r="H137" s="21">
-        <f>IF(OR(J137="",K137="",K137&lt;J137),0,NETWORKDAYS(J137,K137,[1]fESTIVOS!$A$2:$A$53))</f>
-        <v>1</v>
+        <f>IF(OR(J138="",K137="",K137&lt;J138),0,NETWORKDAYS(J138,K137,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>0</v>
       </c>
       <c r="I137" s="87">
         <v>46077</v>
@@ -10954,13 +11036,13 @@
         <v>46077</v>
       </c>
       <c r="M137" s="25">
-        <f ca="1">IF(OR(J137="",AND(L137="",TODAY()&lt;J137),AND(L137&lt;&gt;"",L137&lt;J137)),0,
+        <f ca="1">IF(OR(J138="",AND(L137="",TODAY()&lt;J138),AND(L137&lt;&gt;"",L137&lt;J138)),0,
    IF(L137="",
-      NETWORKDAYS(J137,TODAY(),[1]fESTIVOS!$A$2:$A$53),
-      NETWORKDAYS(J137,L137,[1]fESTIVOS!$A$2:$A$53)
-   )
-)</f>
-        <v>1</v>
+      NETWORKDAYS(J138,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J138,L137,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
       </c>
       <c r="N137" s="84"/>
       <c r="O137" s="84"/>
@@ -10996,7 +11078,7 @@
         <v>100</v>
       </c>
       <c r="H138" s="21">
-        <f>IF(OR(J138="",K138="",K138&lt;J138),0,NETWORKDAYS(J138,K138,[1]fESTIVOS!$A$2:$A$53))</f>
+        <f>IF(OR(J139="",K138="",K138&lt;J139),0,NETWORKDAYS(J139,K138,[1]fESTIVOS!$A$2:$A$53))</f>
         <v>1</v>
       </c>
       <c r="I138" s="87">
@@ -11012,10 +11094,10 @@
         <v>46079</v>
       </c>
       <c r="M138" s="25">
-        <f ca="1">IF(OR(J138="",AND(L138="",TODAY()&lt;J138),AND(L138&lt;&gt;"",L138&lt;J138)),0,
+        <f ca="1">IF(OR(J139="",AND(L138="",TODAY()&lt;J139),AND(L138&lt;&gt;"",L138&lt;J139)),0,
    IF(L138="",
-      NETWORKDAYS(J138,TODAY(),[1]fESTIVOS!$A$2:$A$53),
-      NETWORKDAYS(J138,L138,[1]fESTIVOS!$A$2:$A$53)
+      NETWORKDAYS(J139,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J139,L138,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
         <v>1</v>
@@ -11054,8 +11136,8 @@
         <v>100</v>
       </c>
       <c r="H139" s="21">
-        <f>IF(OR(J139="",K139="",K139&lt;J139),0,NETWORKDAYS(J139,K139,[1]fESTIVOS!$A$2:$A$53))</f>
-        <v>1</v>
+        <f>IF(OR(J140="",K139="",K139&lt;J140),0,NETWORKDAYS(J140,K139,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>0</v>
       </c>
       <c r="I139" s="87">
         <v>46079</v>
@@ -11070,13 +11152,13 @@
         <v>46079</v>
       </c>
       <c r="M139" s="25">
-        <f ca="1">IF(OR(J139="",AND(L139="",TODAY()&lt;J139),AND(L139&lt;&gt;"",L139&lt;J139)),0,
+        <f ca="1">IF(OR(J140="",AND(L139="",TODAY()&lt;J140),AND(L139&lt;&gt;"",L139&lt;J140)),0,
    IF(L139="",
-      NETWORKDAYS(J139,TODAY(),[1]fESTIVOS!$A$2:$A$53),
-      NETWORKDAYS(J139,L139,[1]fESTIVOS!$A$2:$A$53)
-   )
-)</f>
-        <v>1</v>
+      NETWORKDAYS(J140,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J140,L139,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
       </c>
       <c r="N139" s="68"/>
       <c r="O139" s="68"/>
@@ -11112,7 +11194,7 @@
         <v>100</v>
       </c>
       <c r="H140" s="21">
-        <f>IF(OR(J140="",K140="",K140&lt;J140),0,NETWORKDAYS(J140,K140,[1]fESTIVOS!$A$2:$A$53))</f>
+        <f>IF(OR(J141="",K140="",K140&lt;J141),0,NETWORKDAYS(J141,K140,[1]fESTIVOS!$A$2:$A$53))</f>
         <v>1</v>
       </c>
       <c r="I140" s="87">
@@ -11128,10 +11210,10 @@
         <v>46080</v>
       </c>
       <c r="M140" s="25">
-        <f ca="1">IF(OR(J140="",AND(L140="",TODAY()&lt;J140),AND(L140&lt;&gt;"",L140&lt;J140)),0,
+        <f ca="1">IF(OR(J141="",AND(L140="",TODAY()&lt;J141),AND(L140&lt;&gt;"",L140&lt;J141)),0,
    IF(L140="",
-      NETWORKDAYS(J140,TODAY(),[1]fESTIVOS!$A$2:$A$53),
-      NETWORKDAYS(J140,L140,[1]fESTIVOS!$A$2:$A$53)
+      NETWORKDAYS(J141,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J141,L140,[1]fESTIVOS!$A$2:$A$53)
    )
 )</f>
         <v>1</v>
@@ -11170,8 +11252,8 @@
         <v>100</v>
       </c>
       <c r="H141" s="21">
-        <f>IF(OR(J141="",K141="",K141&lt;J141),0,NETWORKDAYS(J141,K141,[1]fESTIVOS!$A$2:$A$53))</f>
-        <v>1</v>
+        <f>IF(OR(J142="",K141="",K141&lt;J142),0,NETWORKDAYS(J142,K141,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>0</v>
       </c>
       <c r="I141" s="87">
         <v>46080</v>
@@ -11186,13 +11268,13 @@
         <v>46080</v>
       </c>
       <c r="M141" s="25">
-        <f ca="1">IF(OR(J141="",AND(L141="",TODAY()&lt;J141),AND(L141&lt;&gt;"",L141&lt;J141)),0,
+        <f ca="1">IF(OR(J142="",AND(L141="",TODAY()&lt;J142),AND(L141&lt;&gt;"",L141&lt;J142)),0,
    IF(L141="",
-      NETWORKDAYS(J141,TODAY(),[1]fESTIVOS!$A$2:$A$53),
-      NETWORKDAYS(J141,L141,[1]fESTIVOS!$A$2:$A$53)
-   )
-)</f>
-        <v>1</v>
+      NETWORKDAYS(J142,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J142,L141,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
       </c>
       <c r="N141" s="68"/>
       <c r="O141" s="68"/>
@@ -11205,25 +11287,367 @@
       </c>
       <c r="S141" s="76"/>
     </row>
-    <row r="142" spans="1:19" ht="29.25" customHeight="1"/>
-    <row r="143" spans="1:19" ht="29.25" customHeight="1"/>
-    <row r="144" spans="1:19" ht="29.25" customHeight="1"/>
-    <row r="145" ht="29.25" customHeight="1"/>
-    <row r="146" ht="29.25" customHeight="1"/>
-    <row r="147" ht="29.25" customHeight="1"/>
-    <row r="148" ht="29.25" customHeight="1"/>
-    <row r="149" ht="29.25" customHeight="1"/>
-    <row r="150" ht="29.25" customHeight="1"/>
-    <row r="151" ht="29.25" customHeight="1"/>
-    <row r="152" ht="29.25" customHeight="1"/>
-    <row r="153" ht="29.25" customHeight="1"/>
-    <row r="154" ht="29.25" customHeight="1"/>
-    <row r="155" ht="29.25" customHeight="1"/>
-    <row r="156" ht="29.25" customHeight="1"/>
-    <row r="157" ht="29.25" customHeight="1"/>
-    <row r="158" ht="29.25" customHeight="1"/>
-    <row r="159" ht="29.25" customHeight="1"/>
-    <row r="160" ht="29.25" customHeight="1"/>
+    <row r="142" spans="1:19" ht="29.25" customHeight="1">
+      <c r="A142" s="80" t="s">
+        <v>19</v>
+      </c>
+      <c r="B142" s="63" t="s">
+        <v>506</v>
+      </c>
+      <c r="C142" s="81" t="s">
+        <v>507</v>
+      </c>
+      <c r="D142" s="92" t="s">
+        <v>508</v>
+      </c>
+      <c r="E142" s="63" t="s">
+        <v>105</v>
+      </c>
+      <c r="F142" s="91" t="s">
+        <v>23</v>
+      </c>
+      <c r="G142" s="83">
+        <v>100</v>
+      </c>
+      <c r="H142" s="21">
+        <f>IF(OR(J143="",K142="",K142&lt;J143),0,NETWORKDAYS(J143,K142,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I142" s="87">
+        <v>46083</v>
+      </c>
+      <c r="J142" s="73">
+        <v>46083</v>
+      </c>
+      <c r="K142" s="73">
+        <v>46084</v>
+      </c>
+      <c r="L142" s="73">
+        <v>46084</v>
+      </c>
+      <c r="M142" s="25">
+        <f ca="1">IF(OR(J143="",AND(L142="",TODAY()&lt;J143),AND(L142&lt;&gt;"",L142&lt;J143)),0,
+   IF(L142="",
+      NETWORKDAYS(J143,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J143,L142,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N142" s="84"/>
+      <c r="O142" s="84"/>
+      <c r="P142" s="85"/>
+      <c r="Q142" s="97" t="s">
+        <v>509</v>
+      </c>
+      <c r="R142" s="71" t="s">
+        <v>25</v>
+      </c>
+      <c r="S142" s="70"/>
+    </row>
+    <row r="143" spans="1:19" ht="29.25" customHeight="1">
+      <c r="A143" s="80" t="s">
+        <v>19</v>
+      </c>
+      <c r="B143" s="63" t="s">
+        <v>510</v>
+      </c>
+      <c r="C143" s="81" t="s">
+        <v>511</v>
+      </c>
+      <c r="D143" s="92" t="s">
+        <v>512</v>
+      </c>
+      <c r="E143" s="63" t="s">
+        <v>105</v>
+      </c>
+      <c r="F143" s="91" t="s">
+        <v>23</v>
+      </c>
+      <c r="G143" s="83">
+        <v>100</v>
+      </c>
+      <c r="H143" s="21">
+        <f>IF(OR(J144="",K143="",K143&lt;J144),0,NETWORKDAYS(J144,K143,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I143" s="87">
+        <v>46085</v>
+      </c>
+      <c r="J143" s="73">
+        <v>46085</v>
+      </c>
+      <c r="K143" s="73">
+        <v>46085</v>
+      </c>
+      <c r="L143" s="73">
+        <v>46085</v>
+      </c>
+      <c r="M143" s="25">
+        <f ca="1">IF(OR(J144="",AND(L143="",TODAY()&lt;J144),AND(L143&lt;&gt;"",L143&lt;J144)),0,
+   IF(L143="",
+      NETWORKDAYS(J144,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J144,L143,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N143" s="84"/>
+      <c r="O143" s="84"/>
+      <c r="P143" s="85"/>
+      <c r="Q143" s="97" t="s">
+        <v>513</v>
+      </c>
+      <c r="R143" s="71" t="s">
+        <v>25</v>
+      </c>
+      <c r="S143" s="70"/>
+    </row>
+    <row r="144" spans="1:19" ht="29.25" customHeight="1">
+      <c r="A144" s="80" t="s">
+        <v>19</v>
+      </c>
+      <c r="B144" s="63" t="s">
+        <v>514</v>
+      </c>
+      <c r="C144" s="81" t="s">
+        <v>515</v>
+      </c>
+      <c r="D144" s="92" t="s">
+        <v>516</v>
+      </c>
+      <c r="E144" s="63" t="s">
+        <v>105</v>
+      </c>
+      <c r="F144" s="91" t="s">
+        <v>23</v>
+      </c>
+      <c r="G144" s="83">
+        <v>100</v>
+      </c>
+      <c r="H144" s="21">
+        <f>IF(OR(J145="",K144="",K144&lt;J145),0,NETWORKDAYS(J145,K144,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>2</v>
+      </c>
+      <c r="I144" s="87">
+        <v>46085</v>
+      </c>
+      <c r="J144" s="73">
+        <v>46085</v>
+      </c>
+      <c r="K144" s="73">
+        <v>46085</v>
+      </c>
+      <c r="L144" s="73">
+        <v>46085</v>
+      </c>
+      <c r="M144" s="25">
+        <f ca="1">IF(OR(J145="",AND(L144="",TODAY()&lt;J145),AND(L144&lt;&gt;"",L144&lt;J145)),0,
+   IF(L144="",
+      NETWORKDAYS(J145,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J145,L144,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>2</v>
+      </c>
+      <c r="N144" s="84"/>
+      <c r="O144" s="84"/>
+      <c r="P144" s="85"/>
+      <c r="Q144" s="97" t="s">
+        <v>517</v>
+      </c>
+      <c r="R144" s="71" t="s">
+        <v>25</v>
+      </c>
+      <c r="S144" s="70"/>
+    </row>
+    <row r="145" spans="1:19" ht="29.25" customHeight="1">
+      <c r="A145" s="88" t="s">
+        <v>19</v>
+      </c>
+      <c r="B145" s="63" t="s">
+        <v>518</v>
+      </c>
+      <c r="C145" s="89" t="s">
+        <v>519</v>
+      </c>
+      <c r="D145" s="93" t="s">
+        <v>520</v>
+      </c>
+      <c r="E145" s="77" t="s">
+        <v>22</v>
+      </c>
+      <c r="F145" s="90" t="s">
+        <v>23</v>
+      </c>
+      <c r="G145" s="78">
+        <v>100</v>
+      </c>
+      <c r="H145" s="21">
+        <f>IF(OR(J146="",K145="",K145&lt;J146),0,NETWORKDAYS(J146,K145,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>1</v>
+      </c>
+      <c r="I145" s="87">
+        <v>46084</v>
+      </c>
+      <c r="J145" s="73">
+        <v>46084</v>
+      </c>
+      <c r="K145" s="73">
+        <v>46086</v>
+      </c>
+      <c r="L145" s="73">
+        <v>46086</v>
+      </c>
+      <c r="M145" s="25">
+        <f ca="1">IF(OR(J146="",AND(L145="",TODAY()&lt;J146),AND(L145&lt;&gt;"",L145&lt;J146)),0,
+   IF(L145="",
+      NETWORKDAYS(J146,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J146,L145,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>1</v>
+      </c>
+      <c r="N145" s="68"/>
+      <c r="O145" s="68"/>
+      <c r="P145" s="69"/>
+      <c r="Q145" s="96" t="s">
+        <v>521</v>
+      </c>
+      <c r="R145" s="79" t="s">
+        <v>25</v>
+      </c>
+      <c r="S145" s="76"/>
+    </row>
+    <row r="146" spans="1:19" ht="29.25" customHeight="1">
+      <c r="A146" s="88" t="s">
+        <v>19</v>
+      </c>
+      <c r="B146" s="63" t="s">
+        <v>522</v>
+      </c>
+      <c r="C146" s="89" t="s">
+        <v>519</v>
+      </c>
+      <c r="D146" s="93" t="s">
+        <v>523</v>
+      </c>
+      <c r="E146" s="77" t="s">
+        <v>22</v>
+      </c>
+      <c r="F146" s="90" t="s">
+        <v>23</v>
+      </c>
+      <c r="G146" s="78">
+        <v>100</v>
+      </c>
+      <c r="H146" s="21">
+        <f>IF(OR(J147="",K146="",K146&lt;J147),0,NETWORKDAYS(J147,K146,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I146" s="87">
+        <v>46086</v>
+      </c>
+      <c r="J146" s="73">
+        <v>46086</v>
+      </c>
+      <c r="K146" s="73">
+        <v>46086</v>
+      </c>
+      <c r="L146" s="73">
+        <v>46086</v>
+      </c>
+      <c r="M146" s="25">
+        <f ca="1">IF(OR(J147="",AND(L146="",TODAY()&lt;J147),AND(L146&lt;&gt;"",L146&lt;J147)),0,
+   IF(L146="",
+      NETWORKDAYS(J147,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J147,L146,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N146" s="68"/>
+      <c r="O146" s="68"/>
+      <c r="P146" s="69"/>
+      <c r="Q146" s="96" t="s">
+        <v>524</v>
+      </c>
+      <c r="R146" s="79" t="s">
+        <v>25</v>
+      </c>
+      <c r="S146" s="76"/>
+    </row>
+    <row r="147" spans="1:19" ht="29.25" customHeight="1">
+      <c r="A147" s="88" t="s">
+        <v>19</v>
+      </c>
+      <c r="B147" s="63" t="s">
+        <v>525</v>
+      </c>
+      <c r="C147" s="89" t="s">
+        <v>519</v>
+      </c>
+      <c r="D147" s="93" t="s">
+        <v>523</v>
+      </c>
+      <c r="E147" s="77" t="s">
+        <v>22</v>
+      </c>
+      <c r="F147" s="90" t="s">
+        <v>23</v>
+      </c>
+      <c r="G147" s="78">
+        <v>100</v>
+      </c>
+      <c r="H147" s="21">
+        <f>IF(OR(J148="",K147="",K147&lt;J148),0,NETWORKDAYS(J148,K147,[1]fESTIVOS!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I147" s="87">
+        <v>46087</v>
+      </c>
+      <c r="J147" s="73">
+        <v>46087</v>
+      </c>
+      <c r="K147" s="73">
+        <v>46087</v>
+      </c>
+      <c r="L147" s="73">
+        <v>46087</v>
+      </c>
+      <c r="M147" s="25">
+        <f ca="1">IF(OR(J148="",AND(L147="",TODAY()&lt;J148),AND(L147&lt;&gt;"",L147&lt;J148)),0,
+   IF(L147="",
+      NETWORKDAYS(J148,TODAY(),[1]fESTIVOS!$A$2:$A$53),
+      NETWORKDAYS(J148,L147,[1]fESTIVOS!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N147" s="68"/>
+      <c r="O147" s="68"/>
+      <c r="P147" s="69"/>
+      <c r="Q147" s="96" t="s">
+        <v>526</v>
+      </c>
+      <c r="R147" s="79" t="s">
+        <v>25</v>
+      </c>
+      <c r="S147" s="76"/>
+    </row>
+    <row r="148" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="149" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="150" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="151" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="152" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="153" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="154" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="155" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="156" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="157" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="158" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="159" spans="1:19" ht="29.25" customHeight="1"/>
+    <row r="160" spans="1:19" ht="29.25" customHeight="1"/>
     <row r="161" ht="29.25" customHeight="1"/>
     <row r="162" ht="29.25" customHeight="1"/>
     <row r="163" ht="29.25" customHeight="1"/>
@@ -12124,18 +12548,24 @@
     <row r="1058" ht="29.25" customHeight="1"/>
     <row r="1059" ht="29.25" customHeight="1"/>
     <row r="1060" ht="29.25" customHeight="1"/>
+    <row r="1061" ht="29.25" customHeight="1"/>
+    <row r="1062" ht="29.25" customHeight="1"/>
+    <row r="1063" ht="29.25" customHeight="1"/>
+    <row r="1064" ht="29.25" customHeight="1"/>
+    <row r="1065" ht="29.25" customHeight="1"/>
+    <row r="1066" ht="29.25" customHeight="1"/>
   </sheetData>
-  <conditionalFormatting sqref="B2:B142">
+  <conditionalFormatting sqref="B2:B148">
     <cfRule type="expression" dxfId="0" priority="2">
-      <formula>COUNTIF($B$2:$B$141,B2)&gt;1</formula>
+      <formula>COUNTIF($B$2:$B$147,B2)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="1" showDropDown="1" sqref="R2:R141"/>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:L141 O2:P141">
+    <dataValidation allowBlank="1" showDropDown="1" sqref="R2:R147"/>
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:L147 O2:P147">
       <formula1>OR(NOT(ISERROR(DATEVALUE(I2))), AND(ISNUMBER(I2), LEFT(CELL("format", I2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F141">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F147">
       <formula1>"FINALIZADO,EN PROCESO,PAUSADO,EN TEST,PENDIENTE,PRUEBAS CLIENTE,PENDIENTE CLIENTE,PRUEBAS IMAGINE,PASO A PRODUCCION"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>